<commit_message>
Fix the sample work plan import for production
The clean sample file showed five errors on production. Three rows named
a "Dig-once repair" combination that only the local database has, and
two named segments that are active locally but not on production
(WL-0206 is inactive, WL-0253 is planned).

The generator now uses no combinations, only single treatments from the
seeded library, and it swaps those two segments for others from the same
condition band. It takes them from the far end of the band so that every
other row keeps the segment production already accepted. The rows are
now 9, 15 and 21 as Spot Repair, 20 on WL-0067 and 31 on WL-0076. Both
files are regenerated.

Migrations: none.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/prisma/sample-data/work-plan-import-2026-2030-with-errors.xlsx
+++ b/prisma/sample-data/work-plan-import-2026-2030-with-errors.xlsx
@@ -96,223 +96,223 @@
     <t>WL-0219</t>
   </si>
   <si>
+    <t>Spot Repair</t>
+  </si>
+  <si>
+    <t>CIP-2026-005 · condition 55</t>
+  </si>
+  <si>
+    <t>WL-0090</t>
+  </si>
+  <si>
+    <t>Lining</t>
+  </si>
+  <si>
+    <t>CIP-2026-006 · condition 55</t>
+  </si>
+  <si>
+    <t>WL-0252</t>
+  </si>
+  <si>
+    <t>CIP-2027-001 · condition 5</t>
+  </si>
+  <si>
+    <t>WL-0229</t>
+  </si>
+  <si>
+    <t>CIP-2027-002 · condition 6</t>
+  </si>
+  <si>
+    <t>WL-0132</t>
+  </si>
+  <si>
+    <t>CIP-2027-003 · condition 37</t>
+  </si>
+  <si>
+    <t>WL-0258</t>
+  </si>
+  <si>
+    <t>CIP-2027-004 · condition 38</t>
+  </si>
+  <si>
+    <t>WL-0200</t>
+  </si>
+  <si>
+    <t>CIP-2027-005 · condition 56</t>
+  </si>
+  <si>
+    <t>WL-0045</t>
+  </si>
+  <si>
+    <t>CIP-2027-006 · condition 56</t>
+  </si>
+  <si>
+    <t>WL-0026</t>
+  </si>
+  <si>
+    <t>Planned</t>
+  </si>
+  <si>
+    <t>CIP-2028-001 · condition 7</t>
+  </si>
+  <si>
+    <t>WL-0190</t>
+  </si>
+  <si>
+    <t>CIP-2028-002 · condition 7</t>
+  </si>
+  <si>
+    <t>WL-0193</t>
+  </si>
+  <si>
+    <t>CIP-2028-003 · condition 38</t>
+  </si>
+  <si>
+    <t>WL-0067</t>
+  </si>
+  <si>
+    <t>CIP-2028-004 · condition 55</t>
+  </si>
+  <si>
+    <t>WL-0166</t>
+  </si>
+  <si>
+    <t>CIP-2028-005 · condition 56</t>
+  </si>
+  <si>
+    <t>WL-0137</t>
+  </si>
+  <si>
+    <t>CIP-2028-006 · condition 56</t>
+  </si>
+  <si>
+    <t>WL-0227</t>
+  </si>
+  <si>
+    <t>CIP-2029-001 · condition 8</t>
+  </si>
+  <si>
+    <t>WL-0064</t>
+  </si>
+  <si>
+    <t>CIP-2029-002 · condition 8</t>
+  </si>
+  <si>
+    <t>WL-0107</t>
+  </si>
+  <si>
+    <t>CIP-2029-003 · condition 38</t>
+  </si>
+  <si>
+    <t>WL-0247</t>
+  </si>
+  <si>
+    <t>CIP-2029-004 · condition 38</t>
+  </si>
+  <si>
+    <t>WL-0127</t>
+  </si>
+  <si>
+    <t>CIP-2029-005 · condition 57</t>
+  </si>
+  <si>
+    <t>WL-0145</t>
+  </si>
+  <si>
+    <t>CIP-2029-006 · condition 57</t>
+  </si>
+  <si>
+    <t>WL-0098</t>
+  </si>
+  <si>
+    <t>CIP-2030-001 · condition 8</t>
+  </si>
+  <si>
+    <t>WL-0164</t>
+  </si>
+  <si>
+    <t>CIP-2030-002 · condition 9</t>
+  </si>
+  <si>
+    <t>WL-0076</t>
+  </si>
+  <si>
+    <t>CIP-2030-003 · condition 55</t>
+  </si>
+  <si>
+    <t>WL-0062</t>
+  </si>
+  <si>
+    <t>CIP-2030-004 · condition 39</t>
+  </si>
+  <si>
+    <t>WL-0099</t>
+  </si>
+  <si>
+    <t>CIP-2030-005 · condition 57</t>
+  </si>
+  <si>
+    <t>WL-0250</t>
+  </si>
+  <si>
+    <t>CIP-2030-006 · condition 57</t>
+  </si>
+  <si>
+    <t>WL-9999</t>
+  </si>
+  <si>
+    <t>Mistake: no such segment</t>
+  </si>
+  <si>
+    <t>Pipe Bursting</t>
+  </si>
+  <si>
+    <t>Mistake: not in the treatment library</t>
+  </si>
+  <si>
+    <t>Mistake: outside a 2026–2030 plan</t>
+  </si>
+  <si>
+    <t>TBD</t>
+  </si>
+  <si>
+    <t>Mistake: cost is not an amount</t>
+  </si>
+  <si>
+    <t>Mistake: programmed after the year it is paid for</t>
+  </si>
+  <si>
+    <t>How to fill in each column</t>
+  </si>
+  <si>
+    <t>Every row is checked before anything is imported, and nothing is written while any row has an error.</t>
+  </si>
+  <si>
+    <t>Column</t>
+  </si>
+  <si>
+    <t>Required</t>
+  </si>
+  <si>
+    <t>What to put</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>The segment's asset ID. It must be an active segment.</t>
+  </si>
+  <si>
+    <t>WL-0058</t>
+  </si>
+  <si>
+    <t>A treatment or a treatment combination, spelled as in the library (see the Treatments sheet). A combination imports as one project. Anything not in the library must be created in Settings first.</t>
+  </si>
+  <si>
     <t>Dig-once repair</t>
-  </si>
-  <si>
-    <t>CIP-2026-005 · condition 55</t>
-  </si>
-  <si>
-    <t>WL-0090</t>
-  </si>
-  <si>
-    <t>Lining</t>
-  </si>
-  <si>
-    <t>CIP-2026-006 · condition 55</t>
-  </si>
-  <si>
-    <t>WL-0252</t>
-  </si>
-  <si>
-    <t>CIP-2027-001 · condition 5</t>
-  </si>
-  <si>
-    <t>WL-0229</t>
-  </si>
-  <si>
-    <t>CIP-2027-002 · condition 6</t>
-  </si>
-  <si>
-    <t>WL-0132</t>
-  </si>
-  <si>
-    <t>CIP-2027-003 · condition 37</t>
-  </si>
-  <si>
-    <t>WL-0258</t>
-  </si>
-  <si>
-    <t>CIP-2027-004 · condition 38</t>
-  </si>
-  <si>
-    <t>WL-0200</t>
-  </si>
-  <si>
-    <t>CIP-2027-005 · condition 56</t>
-  </si>
-  <si>
-    <t>WL-0045</t>
-  </si>
-  <si>
-    <t>CIP-2027-006 · condition 56</t>
-  </si>
-  <si>
-    <t>WL-0026</t>
-  </si>
-  <si>
-    <t>Planned</t>
-  </si>
-  <si>
-    <t>CIP-2028-001 · condition 7</t>
-  </si>
-  <si>
-    <t>WL-0190</t>
-  </si>
-  <si>
-    <t>CIP-2028-002 · condition 7</t>
-  </si>
-  <si>
-    <t>WL-0193</t>
-  </si>
-  <si>
-    <t>CIP-2028-003 · condition 38</t>
-  </si>
-  <si>
-    <t>WL-0206</t>
-  </si>
-  <si>
-    <t>CIP-2028-004 · condition 38</t>
-  </si>
-  <si>
-    <t>WL-0166</t>
-  </si>
-  <si>
-    <t>CIP-2028-005 · condition 56</t>
-  </si>
-  <si>
-    <t>WL-0137</t>
-  </si>
-  <si>
-    <t>CIP-2028-006 · condition 56</t>
-  </si>
-  <si>
-    <t>WL-0227</t>
-  </si>
-  <si>
-    <t>CIP-2029-001 · condition 8</t>
-  </si>
-  <si>
-    <t>WL-0064</t>
-  </si>
-  <si>
-    <t>CIP-2029-002 · condition 8</t>
-  </si>
-  <si>
-    <t>WL-0107</t>
-  </si>
-  <si>
-    <t>CIP-2029-003 · condition 38</t>
-  </si>
-  <si>
-    <t>WL-0247</t>
-  </si>
-  <si>
-    <t>CIP-2029-004 · condition 38</t>
-  </si>
-  <si>
-    <t>WL-0127</t>
-  </si>
-  <si>
-    <t>Spot Repair</t>
-  </si>
-  <si>
-    <t>CIP-2029-005 · condition 57</t>
-  </si>
-  <si>
-    <t>WL-0145</t>
-  </si>
-  <si>
-    <t>CIP-2029-006 · condition 57</t>
-  </si>
-  <si>
-    <t>WL-0098</t>
-  </si>
-  <si>
-    <t>CIP-2030-001 · condition 8</t>
-  </si>
-  <si>
-    <t>WL-0164</t>
-  </si>
-  <si>
-    <t>CIP-2030-002 · condition 9</t>
-  </si>
-  <si>
-    <t>WL-0253</t>
-  </si>
-  <si>
-    <t>CIP-2030-003 · condition 39</t>
-  </si>
-  <si>
-    <t>WL-0062</t>
-  </si>
-  <si>
-    <t>CIP-2030-004 · condition 39</t>
-  </si>
-  <si>
-    <t>WL-0099</t>
-  </si>
-  <si>
-    <t>CIP-2030-005 · condition 57</t>
-  </si>
-  <si>
-    <t>WL-0250</t>
-  </si>
-  <si>
-    <t>CIP-2030-006 · condition 57</t>
-  </si>
-  <si>
-    <t>WL-9999</t>
-  </si>
-  <si>
-    <t>Mistake: no such segment</t>
-  </si>
-  <si>
-    <t>Pipe Bursting</t>
-  </si>
-  <si>
-    <t>Mistake: not in the treatment library</t>
-  </si>
-  <si>
-    <t>Mistake: outside a 2026–2030 plan</t>
-  </si>
-  <si>
-    <t>TBD</t>
-  </si>
-  <si>
-    <t>Mistake: cost is not an amount</t>
-  </si>
-  <si>
-    <t>Mistake: programmed after the year it is paid for</t>
-  </si>
-  <si>
-    <t>How to fill in each column</t>
-  </si>
-  <si>
-    <t>Every row is checked before anything is imported, and nothing is written while any row has an error.</t>
-  </si>
-  <si>
-    <t>Column</t>
-  </si>
-  <si>
-    <t>Required</t>
-  </si>
-  <si>
-    <t>What to put</t>
-  </si>
-  <si>
-    <t>Example</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>The segment's asset ID. It must be an active segment.</t>
-  </si>
-  <si>
-    <t>WL-0058</t>
-  </si>
-  <si>
-    <t>A treatment or a treatment combination, spelled as in the library (see the Treatments sheet). A combination imports as one project. Anything not in the library must be created in Settings first.</t>
   </si>
   <si>
     <t>The year the money is spent. It must fall inside the plan. Without the two columns below, it is also the year the work is decided and built.</t>
@@ -1020,7 +1020,7 @@
         <v>2026</v>
       </c>
       <c r="F9" s="1">
-        <v>30000</v>
+        <v>15000</v>
       </c>
       <c r="G9" t="s">
         <v>13</v>
@@ -1326,7 +1326,7 @@
         <v>2028</v>
       </c>
       <c r="F21" s="1">
-        <v>30000</v>
+        <v>15000</v>
       </c>
       <c r="G21" t="s">
         <v>45</v>
@@ -1474,7 +1474,7 @@
         <v>65</v>
       </c>
       <c r="B27" t="s">
-        <v>66</v>
+        <v>27</v>
       </c>
       <c r="C27">
         <v>2029</v>
@@ -1487,12 +1487,12 @@
         <v>18</v>
       </c>
       <c r="I27" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B28" t="s">
         <v>30</v>
@@ -1508,12 +1508,12 @@
         <v>22</v>
       </c>
       <c r="I28" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B29" t="s">
         <v>12</v>
@@ -1537,12 +1537,12 @@
         <v>14</v>
       </c>
       <c r="I29" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B30" t="s">
         <v>12</v>
@@ -1564,12 +1564,12 @@
         <v>18</v>
       </c>
       <c r="I30" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B31" t="s">
         <v>21</v>
@@ -1591,12 +1591,12 @@
         <v>22</v>
       </c>
       <c r="I31" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B32" t="s">
         <v>21</v>
@@ -1618,12 +1618,12 @@
         <v>14</v>
       </c>
       <c r="I32" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B33" t="s">
         <v>30</v>
@@ -1641,12 +1641,12 @@
         <v>18</v>
       </c>
       <c r="I33" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B34" t="s">
         <v>30</v>
@@ -1662,22 +1662,22 @@
         <v>22</v>
       </c>
       <c r="I34" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B35" t="s">
-        <v>66</v>
+        <v>27</v>
       </c>
       <c r="C35">
         <v>2027</v>
       </c>
       <c r="F35" s="1"/>
       <c r="I35" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -1685,14 +1685,14 @@
         <v>11</v>
       </c>
       <c r="B36" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C36">
         <v>2028</v>
       </c>
       <c r="F36" s="1"/>
       <c r="I36" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
@@ -1700,14 +1700,14 @@
         <v>16</v>
       </c>
       <c r="B37" t="s">
-        <v>66</v>
+        <v>27</v>
       </c>
       <c r="C37">
         <v>2034</v>
       </c>
       <c r="F37" s="1"/>
       <c r="I37" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
@@ -1715,16 +1715,16 @@
         <v>20</v>
       </c>
       <c r="B38" t="s">
-        <v>66</v>
+        <v>27</v>
       </c>
       <c r="C38">
         <v>2029</v>
       </c>
       <c r="F38" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="I38" t="s">
         <v>87</v>
-      </c>
-      <c r="I38" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="F39" s="1"/>
       <c r="I39" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -1769,7 +1769,7 @@
   <sheetData>
     <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1777,7 +1777,7 @@
     </row>
     <row r="2" spans="1:4" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B2" s="4"/>
       <c r="C2" s="4"/>
@@ -1785,16 +1785,16 @@
     </row>
     <row r="4" spans="1:4" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="D4" s="6" t="s">
         <v>94</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1802,13 +1802,13 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C5" t="s">
         <v>96</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>97</v>
-      </c>
-      <c r="D5" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1816,13 +1816,13 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D6" t="s">
         <v>99</v>
-      </c>
-      <c r="D6" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1830,7 +1830,7 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C7" t="s">
         <v>100</v>
@@ -2086,7 +2086,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>66</v>
+        <v>27</v>
       </c>
       <c r="B15" t="s">
         <v>3</v>
@@ -2119,7 +2119,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>99</v>
       </c>
       <c r="B18" t="s">
         <v>134</v>

</xml_diff>